<commit_message>
feat: adicionar campo opcional de matricula no formulario, planilha e portal de turmas
</commit_message>
<xml_diff>
--- a/public/modelo-importacao-turma.xlsx
+++ b/public/modelo-importacao-turma.xlsx
@@ -439,6 +439,7 @@
   <x:cols>
     <x:col min="1" max="1" width="42" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="24" customHeight="1">
@@ -448,6 +449,9 @@
       <x:c r="B1" s="8" t="str">
         <x:v>CPF</x:v>
       </x:c>
+      <x:c r="C1" s="8" t="str">
+        <x:v>Matrícula</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="22" customHeight="1">
       <x:c r="A2" s="23"/>

</xml_diff>